<commit_message>
Adiciona comparativo de tabela de distribuidor e cotação por embalagem
- comparar_tabela.py cruza o CSV de preços do distribuidor com a Lista de
  Compra por EAN, comparando pela embalagem de compra (Custo un x Un/Cx).
- Modelo de cotação passa a pedir quantidade e preço por embalagem (Caixas),
  pois o EAN da lista é o da embalagem vendida pelo distribuidor (ex.: display).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PaiAv9p4wTkzCU979abHNX
</commit_message>
<xml_diff>
--- a/cotacoes/Cotacao_Rocha_20260925.xlsx
+++ b/cotacoes/Cotacao_Rocha_20260925.xlsx
@@ -658,7 +658,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>• Cada linha é um EAN. Informe o PREÇO UNITÁRIO LÍQUIDO (já com desconto e impostos/ST), por unidade. Ex.: 12,34</t>
+          <t>• Cada linha é um EAN. Informe o PREÇO LÍQUIDO (já com desconto e impostos/ST) da embalagem que o EAN representa (caixa, display etc.). Ex.: 12,34</t>
         </is>
       </c>
     </row>
@@ -704,17 +704,17 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Qtde (un)</t>
+          <t>Qtde (emb.)</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Preço unit. líquido (R$)</t>
+          <t>Preço líquido por emb. (R$)</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>Qtde disponível (un)</t>
+          <t>Qtde disponível (emb.)</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="F27" s="9" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="G27" s="12" t="n"/>
       <c r="H27" s="13" t="n"/>
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="F28" s="9" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="G28" s="12" t="n"/>
       <c r="H28" s="13" t="n"/>
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="F29" s="9" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="G29" s="12" t="n"/>
       <c r="H29" s="13" t="n"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="F30" s="9" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="G30" s="12" t="n"/>
       <c r="H30" s="13" t="n"/>
@@ -1279,7 +1279,7 @@
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="G31" s="12" t="n"/>
       <c r="H31" s="13" t="n"/>
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="G32" s="12" t="n"/>
       <c r="H32" s="13" t="n"/>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="F48" s="9" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="G48" s="12" t="n"/>
       <c r="H48" s="13" t="n"/>
@@ -2335,7 +2335,7 @@
         </is>
       </c>
       <c r="F63" s="15" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G63" s="12" t="n"/>
       <c r="H63" s="13" t="n"/>
@@ -2368,7 +2368,7 @@
         </is>
       </c>
       <c r="F64" s="15" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G64" s="12" t="n"/>
       <c r="H64" s="13" t="n"/>
@@ -2698,7 +2698,7 @@
         </is>
       </c>
       <c r="F74" s="9" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G74" s="12" t="n"/>
       <c r="H74" s="13" t="n"/>
@@ -2731,7 +2731,7 @@
         </is>
       </c>
       <c r="F75" s="15" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="G75" s="12" t="n"/>
       <c r="H75" s="13" t="n"/>
@@ -2764,7 +2764,7 @@
         </is>
       </c>
       <c r="F76" s="15" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="G76" s="12" t="n"/>
       <c r="H76" s="13" t="n"/>
@@ -3028,7 +3028,7 @@
         </is>
       </c>
       <c r="F84" s="15" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G84" s="12" t="n"/>
       <c r="H84" s="13" t="n"/>
@@ -3061,7 +3061,7 @@
         </is>
       </c>
       <c r="F85" s="15" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G85" s="12" t="n"/>
       <c r="H85" s="13" t="n"/>
@@ -3490,7 +3490,7 @@
         </is>
       </c>
       <c r="F98" s="15" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="G98" s="12" t="n"/>
       <c r="H98" s="13" t="n"/>
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="F99" s="15" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="G99" s="12" t="n"/>
       <c r="H99" s="13" t="n"/>
@@ -3556,7 +3556,7 @@
         </is>
       </c>
       <c r="F100" s="9" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="G100" s="12" t="n"/>
       <c r="H100" s="13" t="n"/>
@@ -4678,7 +4678,7 @@
         </is>
       </c>
       <c r="F134" s="9" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="G134" s="12" t="n"/>
       <c r="H134" s="13" t="n"/>
@@ -4711,7 +4711,7 @@
         </is>
       </c>
       <c r="F135" s="9" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="G135" s="12" t="n"/>
       <c r="H135" s="13" t="n"/>
@@ -4843,7 +4843,7 @@
         </is>
       </c>
       <c r="F139" s="9" t="n">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="G139" s="12" t="n"/>
       <c r="H139" s="13" t="n"/>
@@ -4876,7 +4876,7 @@
         </is>
       </c>
       <c r="F140" s="9" t="n">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="G140" s="12" t="n"/>
       <c r="H140" s="13" t="n"/>
@@ -6972,7 +6972,7 @@
         </is>
       </c>
       <c r="F204" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G204" s="12" t="n"/>
       <c r="H204" s="13" t="n"/>
@@ -7071,7 +7071,7 @@
         </is>
       </c>
       <c r="F207" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G207" s="12" t="n"/>
       <c r="H207" s="13" t="n"/>
@@ -7104,7 +7104,7 @@
         </is>
       </c>
       <c r="F208" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G208" s="12" t="n"/>
       <c r="H208" s="13" t="n"/>
@@ -7731,7 +7731,7 @@
         </is>
       </c>
       <c r="F227" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G227" s="12" t="n"/>
       <c r="H227" s="13" t="n"/>
@@ -8882,7 +8882,7 @@
         </is>
       </c>
       <c r="F262" s="15" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="G262" s="12" t="n"/>
       <c r="H262" s="13" t="n"/>
@@ -8915,7 +8915,7 @@
         </is>
       </c>
       <c r="F263" s="15" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="G263" s="12" t="n"/>
       <c r="H263" s="13" t="n"/>
@@ -9179,7 +9179,7 @@
         </is>
       </c>
       <c r="F271" s="15" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="G271" s="12" t="n"/>
       <c r="H271" s="13" t="n"/>
@@ -9831,7 +9831,7 @@
         </is>
       </c>
       <c r="F291" s="15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G291" s="12" t="n"/>
       <c r="H291" s="13" t="n"/>
@@ -9963,7 +9963,7 @@
         </is>
       </c>
       <c r="F295" s="15" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G295" s="12" t="n"/>
       <c r="H295" s="13" t="n"/>
@@ -9996,7 +9996,7 @@
         </is>
       </c>
       <c r="F296" s="15" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G296" s="12" t="n"/>
       <c r="H296" s="13" t="n"/>
@@ -10062,7 +10062,7 @@
         </is>
       </c>
       <c r="F298" s="15" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="G298" s="12" t="n"/>
       <c r="H298" s="13" t="n"/>
@@ -10095,7 +10095,7 @@
         </is>
       </c>
       <c r="F299" s="15" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="G299" s="12" t="n"/>
       <c r="H299" s="13" t="n"/>
@@ -10421,7 +10421,7 @@
         </is>
       </c>
       <c r="F309" s="15" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="G309" s="12" t="n"/>
       <c r="H309" s="13" t="n"/>
@@ -10487,7 +10487,7 @@
         </is>
       </c>
       <c r="F311" s="15" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G311" s="12" t="n"/>
       <c r="H311" s="13" t="n"/>
@@ -10978,7 +10978,7 @@
         </is>
       </c>
       <c r="F326" s="15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G326" s="12" t="n"/>
       <c r="H326" s="13" t="n"/>
@@ -11275,7 +11275,7 @@
         </is>
       </c>
       <c r="F335" s="15" t="n">
-        <v>150</v>
+        <v>15</v>
       </c>
       <c r="G335" s="12" t="n"/>
       <c r="H335" s="13" t="n"/>
@@ -11832,7 +11832,7 @@
         </is>
       </c>
       <c r="F352" s="9" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G352" s="12" t="n"/>
       <c r="H352" s="13" t="n"/>
@@ -11865,7 +11865,7 @@
         </is>
       </c>
       <c r="F353" s="9" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G353" s="12" t="n"/>
       <c r="H353" s="13" t="n"/>
@@ -11898,7 +11898,7 @@
         </is>
       </c>
       <c r="F354" s="15" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="G354" s="12" t="n"/>
       <c r="H354" s="13" t="n"/>
@@ -11931,7 +11931,7 @@
         </is>
       </c>
       <c r="F355" s="15" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="G355" s="12" t="n"/>
       <c r="H355" s="13" t="n"/>
@@ -11964,7 +11964,7 @@
         </is>
       </c>
       <c r="F356" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G356" s="12" t="n"/>
       <c r="H356" s="13" t="n"/>
@@ -11997,7 +11997,7 @@
         </is>
       </c>
       <c r="F357" s="15" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G357" s="12" t="n"/>
       <c r="H357" s="13" t="n"/>
@@ -13152,7 +13152,7 @@
         </is>
       </c>
       <c r="F392" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G392" s="12" t="n"/>
       <c r="H392" s="13" t="n"/>
@@ -13713,7 +13713,7 @@
         </is>
       </c>
       <c r="F409" s="15" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G409" s="12" t="n"/>
       <c r="H409" s="13" t="n"/>
@@ -13746,7 +13746,7 @@
         </is>
       </c>
       <c r="F410" s="15" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G410" s="12" t="n"/>
       <c r="H410" s="13" t="n"/>
@@ -14600,7 +14600,7 @@
         </is>
       </c>
       <c r="F436" s="9" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="G436" s="12" t="n"/>
       <c r="H436" s="13" t="n"/>
@@ -14633,7 +14633,7 @@
         </is>
       </c>
       <c r="F437" s="9" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="G437" s="12" t="n"/>
       <c r="H437" s="13" t="n"/>
@@ -15937,7 +15937,7 @@
         </is>
       </c>
       <c r="F477" s="9" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G477" s="12" t="n"/>
       <c r="H477" s="13" t="n"/>
@@ -16428,7 +16428,7 @@
         </is>
       </c>
       <c r="F492" s="9" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G492" s="12" t="n"/>
       <c r="H492" s="13" t="n"/>
@@ -16758,7 +16758,7 @@
         </is>
       </c>
       <c r="F502" s="9" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="G502" s="12" t="n"/>
       <c r="H502" s="13" t="n"/>
@@ -16791,7 +16791,7 @@
         </is>
       </c>
       <c r="F503" s="9" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="G503" s="12" t="n"/>
       <c r="H503" s="13" t="n"/>
@@ -18301,7 +18301,7 @@
         </is>
       </c>
       <c r="F549" s="15" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G549" s="12" t="n"/>
       <c r="H549" s="13" t="n"/>
@@ -19283,7 +19283,7 @@
         </is>
       </c>
       <c r="F579" s="15" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="G579" s="12" t="n"/>
       <c r="H579" s="13" t="n"/>
@@ -19943,7 +19943,7 @@
         </is>
       </c>
       <c r="F599" s="15" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="G599" s="12" t="n"/>
       <c r="H599" s="13" t="n"/>
@@ -19976,7 +19976,7 @@
         </is>
       </c>
       <c r="F600" s="15" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="G600" s="12" t="n"/>
       <c r="H600" s="13" t="n"/>
@@ -20595,7 +20595,7 @@
         </is>
       </c>
       <c r="F619" s="9" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G619" s="12" t="n"/>
       <c r="H619" s="13" t="n"/>
@@ -21647,7 +21647,7 @@
         </is>
       </c>
       <c r="F651" s="9" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G651" s="12" t="n"/>
       <c r="H651" s="13" t="n"/>
@@ -21680,7 +21680,7 @@
         </is>
       </c>
       <c r="F652" s="9" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G652" s="12" t="n"/>
       <c r="H652" s="13" t="n"/>
@@ -22208,7 +22208,7 @@
         </is>
       </c>
       <c r="F668" s="9" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G668" s="12" t="n"/>
       <c r="H668" s="13" t="n"/>
@@ -22241,7 +22241,7 @@
         </is>
       </c>
       <c r="F669" s="9" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G669" s="12" t="n"/>
       <c r="H669" s="13" t="n"/>
@@ -22864,7 +22864,7 @@
         </is>
       </c>
       <c r="F688" s="15" t="n">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="G688" s="12" t="n"/>
       <c r="H688" s="13" t="n"/>
@@ -22897,7 +22897,7 @@
         </is>
       </c>
       <c r="F689" s="9" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="G689" s="12" t="n"/>
       <c r="H689" s="13" t="n"/>
@@ -22930,7 +22930,7 @@
         </is>
       </c>
       <c r="F690" s="9" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="G690" s="12" t="n"/>
       <c r="H690" s="13" t="n"/>
@@ -22996,7 +22996,7 @@
         </is>
       </c>
       <c r="F692" s="9" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G692" s="12" t="n"/>
       <c r="H692" s="13" t="n"/>
@@ -23029,7 +23029,7 @@
         </is>
       </c>
       <c r="F693" s="15" t="n">
-        <v>210</v>
+        <v>7</v>
       </c>
       <c r="G693" s="12" t="n"/>
       <c r="H693" s="13" t="n"/>
@@ -23062,7 +23062,7 @@
         </is>
       </c>
       <c r="F694" s="15" t="n">
-        <v>210</v>
+        <v>7</v>
       </c>
       <c r="G694" s="12" t="n"/>
       <c r="H694" s="13" t="n"/>
@@ -23095,7 +23095,7 @@
         </is>
       </c>
       <c r="F695" s="9" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G695" s="12" t="n"/>
       <c r="H695" s="13" t="n"/>
@@ -23128,7 +23128,7 @@
         </is>
       </c>
       <c r="F696" s="9" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G696" s="12" t="n"/>
       <c r="H696" s="13" t="n"/>
@@ -23953,7 +23953,7 @@
         </is>
       </c>
       <c r="F721" s="9" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G721" s="12" t="n"/>
       <c r="H721" s="13" t="n"/>
@@ -23986,7 +23986,7 @@
         </is>
       </c>
       <c r="F722" s="9" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G722" s="12" t="n"/>
       <c r="H722" s="13" t="n"/>
@@ -24382,7 +24382,7 @@
         </is>
       </c>
       <c r="F734" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G734" s="12" t="n"/>
       <c r="H734" s="13" t="n"/>
@@ -24844,7 +24844,7 @@
         </is>
       </c>
       <c r="F748" s="9" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G748" s="12" t="n"/>
       <c r="H748" s="13" t="n"/>
@@ -24877,7 +24877,7 @@
         </is>
       </c>
       <c r="F749" s="9" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G749" s="12" t="n"/>
       <c r="H749" s="13" t="n"/>
@@ -25232,7 +25232,7 @@
         </is>
       </c>
       <c r="F760" s="15" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G760" s="12" t="n"/>
       <c r="H760" s="13" t="n"/>
@@ -25265,7 +25265,7 @@
         </is>
       </c>
       <c r="F761" s="15" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G761" s="12" t="n"/>
       <c r="H761" s="13" t="n"/>
@@ -25859,7 +25859,7 @@
         </is>
       </c>
       <c r="F779" s="9" t="n">
-        <v>54</v>
+        <v>9</v>
       </c>
       <c r="G779" s="12" t="n"/>
       <c r="H779" s="13" t="n"/>
@@ -25892,7 +25892,7 @@
         </is>
       </c>
       <c r="F780" s="9" t="n">
-        <v>54</v>
+        <v>9</v>
       </c>
       <c r="G780" s="12" t="n"/>
       <c r="H780" s="13" t="n"/>
@@ -25925,7 +25925,7 @@
         </is>
       </c>
       <c r="F781" s="15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G781" s="12" t="n"/>
       <c r="H781" s="13" t="n"/>
@@ -25958,7 +25958,7 @@
         </is>
       </c>
       <c r="F782" s="15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G782" s="12" t="n"/>
       <c r="H782" s="13" t="n"/>
@@ -25991,7 +25991,7 @@
         </is>
       </c>
       <c r="F783" s="9" t="n">
-        <v>96</v>
+        <v>8</v>
       </c>
       <c r="G783" s="12" t="n"/>
       <c r="H783" s="13" t="n"/>
@@ -26024,7 +26024,7 @@
         </is>
       </c>
       <c r="F784" s="9" t="n">
-        <v>96</v>
+        <v>8</v>
       </c>
       <c r="G784" s="12" t="n"/>
       <c r="H784" s="13" t="n"/>
@@ -26057,7 +26057,7 @@
         </is>
       </c>
       <c r="F785" s="15" t="n">
-        <v>336</v>
+        <v>14</v>
       </c>
       <c r="G785" s="12" t="n"/>
       <c r="H785" s="13" t="n"/>
@@ -26090,7 +26090,7 @@
         </is>
       </c>
       <c r="F786" s="15" t="n">
-        <v>336</v>
+        <v>14</v>
       </c>
       <c r="G786" s="12" t="n"/>
       <c r="H786" s="13" t="n"/>
@@ -26123,7 +26123,7 @@
         </is>
       </c>
       <c r="F787" s="15" t="n">
-        <v>336</v>
+        <v>14</v>
       </c>
       <c r="G787" s="12" t="n"/>
       <c r="H787" s="13" t="n"/>
@@ -26156,7 +26156,7 @@
         </is>
       </c>
       <c r="F788" s="15" t="n">
-        <v>336</v>
+        <v>14</v>
       </c>
       <c r="G788" s="12" t="n"/>
       <c r="H788" s="13" t="n"/>
@@ -26189,7 +26189,7 @@
         </is>
       </c>
       <c r="F789" s="9" t="n">
-        <v>250</v>
+        <v>5</v>
       </c>
       <c r="G789" s="12" t="n"/>
       <c r="H789" s="13" t="n"/>
@@ -26552,7 +26552,7 @@
         </is>
       </c>
       <c r="F800" s="9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G800" s="12" t="n"/>
       <c r="H800" s="13" t="n"/>
@@ -26585,7 +26585,7 @@
         </is>
       </c>
       <c r="F801" s="15" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G801" s="12" t="n"/>
       <c r="H801" s="13" t="n"/>
@@ -26618,7 +26618,7 @@
         </is>
       </c>
       <c r="F802" s="15" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G802" s="12" t="n"/>
       <c r="H802" s="13" t="n"/>
@@ -26651,7 +26651,7 @@
         </is>
       </c>
       <c r="F803" s="9" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="G803" s="12" t="n"/>
       <c r="H803" s="13" t="n"/>
@@ -26684,7 +26684,7 @@
         </is>
       </c>
       <c r="F804" s="9" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="G804" s="12" t="n"/>
       <c r="H804" s="13" t="n"/>
@@ -26717,7 +26717,7 @@
         </is>
       </c>
       <c r="F805" s="9" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="G805" s="12" t="n"/>
       <c r="H805" s="13" t="n"/>
@@ -26750,7 +26750,7 @@
         </is>
       </c>
       <c r="F806" s="9" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="G806" s="12" t="n"/>
       <c r="H806" s="13" t="n"/>
@@ -27031,10 +27031,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G15:G813" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor inválido" error="Informe apenas o preço unitário em número (ex.: 12,34)." type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="G15:G813" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor inválido" error="Informe apenas o preço em número (ex.: 12,34)." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="H15:H813" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor inválido" error="Informe a quantidade em unidades inteiras." type="whole" operator="greaterThanOrEqual">
+    <dataValidation sqref="H15:H813" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Valor inválido" error="Informe a quantidade em número inteiro de embalagens." type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>